<commit_message>
fix: update RO block dropdown booth counts in entry console (Semari 76, Lasadiya 74, Salumbar 77, Sarada 78, Jhallara 83) and sync Excel ZP ward contributing counts
</commit_message>
<xml_diff>
--- a/Salumber_Consolidated_Master_Elections_2026.xlsx
+++ b/Salumber_Consolidated_Master_Elections_2026.xlsx
@@ -32712,7 +32712,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Semari (21)</t>
+          <t>Semari (24)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -32741,7 +32741,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Semari (25)</t>
+          <t>Semari (26)</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -32770,7 +32770,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Semari (23)</t>
+          <t>Semari (26)</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -33031,7 +33031,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Lasadiya (28)</t>
+          <t>Lasadiya (29)</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">

</xml_diff>